<commit_message>
docs: 更新 IG 網頁（0 errors, 0 warnings）
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-AA12Model.xlsx
+++ b/docs/StructureDefinition-AA12Model.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.4.1</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-28T23:13:53+08:00</t>
+    <t>2026-03-01T19:25:35+08:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>